<commit_message>
test if removing ramp up limit or
or impose higher multiplior for grid-storage works for generation mix
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_zAK_fixes.xlsx
+++ b/SuppXLS/Scen_zAK_fixes.xlsx
@@ -2006,7 +2006,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B5:N85"/>
+  <dimension ref="B3:N85"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="35.6363636363636" customWidth="1"/>
@@ -2014,10 +2014,12 @@
     <col min="5" max="5" width="10.1818181818182" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="3" spans="2:14">
+      <c r="C3" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="5" spans="2:14">
-      <c r="C5" s="8" t="s">
-        <v>23</v>
-      </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
       <c r="F5" s="10"/>

</xml_diff>

<commit_message>
EN_.. starts in 2020
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_zAK_fixes.xlsx
+++ b/SuppXLS/Scen_zAK_fixes.xlsx
@@ -775,11 +775,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="0"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
@@ -794,6 +789,11 @@
     <font>
       <sz val="9"/>
       <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
       <charset val="0"/>
     </font>
   </fonts>
@@ -2338,7 +2338,7 @@
         <v>45</v>
       </c>
       <c r="E27" s="20">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="F27" s="10"/>
     </row>

</xml_diff>

<commit_message>
grid storage lower than ...
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_zAK_fixes.xlsx
+++ b/SuppXLS/Scen_zAK_fixes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13120" windowHeight="8980" firstSheet="1" activeTab="4"/>
+    <workbookView windowWidth="19200" windowHeight="8710" firstSheet="4" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="INS" sheetId="2" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="ROR_has_no_regulation_cap" sheetId="10" r:id="rId4"/>
     <sheet name="Ramp_rate_constraints" sheetId="11" r:id="rId5"/>
     <sheet name="Growth_rate" sheetId="12" r:id="rId6"/>
+    <sheet name="Peak_demand_limit_battery" sheetId="13" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="IQ_FWD_Q" hidden="1">501</definedName>
@@ -242,8 +243,40 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>xli9</author>
+  </authors>
+  <commentList>
+    <comment ref="M20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>xli9:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Bca the capacity unit is GWh</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="137">
   <si>
     <t>~TFM_UPD</t>
   </si>
@@ -564,6 +597,96 @@
   </si>
   <si>
     <t>Tra_EV_Batt-NMC811_fromrecy</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy8</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt</t>
+  </si>
+  <si>
+    <t>2020, 2150</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy9</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt_LMO</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy10</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt_NCA</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy11</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt_NMC111</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy12</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt_NMC532</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy13</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt_NMC622</t>
+  </si>
+  <si>
+    <t>UC_Grow_Recy14</t>
+  </si>
+  <si>
+    <t>EN_STG_4hBatt_NMC811</t>
+  </si>
+  <si>
+    <t>~UC_Sets: R_E: AllRegions</t>
+  </si>
+  <si>
+    <t>~UC_T: UP</t>
+  </si>
+  <si>
+    <t>Pset_CI</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>UC_FLO</t>
+  </si>
+  <si>
+    <t>UC_COMPRD</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS</t>
+  </si>
+  <si>
+    <t>UC_RHSRTS~0</t>
+  </si>
+  <si>
+    <t>UCE_Min-DispatchablePrd</t>
+  </si>
+  <si>
+    <t>ELE,CHP</t>
+  </si>
+  <si>
+    <t>E*</t>
+  </si>
+  <si>
+    <t>ELCSPV</t>
+  </si>
+  <si>
+    <t>Discharge of batteries should lower than a level</t>
+  </si>
+  <si>
+    <t>AuxStoOUT</t>
+  </si>
+  <si>
+    <t>ELCWIN</t>
   </si>
 </sst>
 </file>
@@ -784,7 +907,6 @@
       <charset val="0"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="0"/>
@@ -795,12 +917,13 @@
       <charset val="0"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="0"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -809,7 +932,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -822,12 +957,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1018,7 +1147,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1027,40 +1156,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFDEE2E6"/>
-      </left>
+      <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
+      <top style="thick">
+        <color rgb="FFFC8462"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
+      <bottom style="thick">
+        <color rgb="FFFC8462"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1185,7 +1288,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1197,124 +1300,127 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1322,30 +1428,34 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="49" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="49" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="49" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="52" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="52" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="52" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="52" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="52" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="53">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1879,7 +1989,7 @@
       <c r="E21" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="2">
         <v>0.5</v>
       </c>
       <c r="G21" t="str">
@@ -1936,7 +2046,7 @@
       </c>
     </row>
     <row r="4" ht="16" spans="1:11">
-      <c r="A4" s="3"/>
+      <c r="A4" s="6"/>
     </row>
     <row r="7" spans="1:11">
       <c r="D7" t="s">
@@ -1993,10 +2103,10 @@
       <c r="H10">
         <v>0.48</v>
       </c>
-      <c r="K10" s="23"/>
+      <c r="K10" s="28"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="K11" s="23"/>
+      <c r="K11" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2017,12 +2127,12 @@
   </cols>
   <sheetData>
     <row r="5" spans="2:13">
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="10"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="2:13">
       <c r="B6" t="s">
@@ -2037,19 +2147,19 @@
       <c r="E6" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="11"/>
+      <c r="K6" s="18"/>
     </row>
     <row r="7" spans="2:13">
       <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="19">
         <v>10</v>
       </c>
     </row>
@@ -2057,29 +2167,29 @@
       <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="19">
         <v>7</v>
       </c>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
     </row>
     <row r="9" ht="16" spans="2:13">
       <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="19">
         <v>10</v>
       </c>
     </row>
@@ -2087,29 +2197,29 @@
       <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="19">
         <v>8</v>
       </c>
-      <c r="K10" s="13"/>
-      <c r="L10" s="14"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="21"/>
     </row>
     <row r="11" ht="16" spans="2:13">
       <c r="B11" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="17">
         <v>1.5</v>
       </c>
     </row>
@@ -2117,13 +2227,13 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="17">
         <v>1.5</v>
       </c>
     </row>
@@ -2131,13 +2241,13 @@
       <c r="B13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="7">
         <v>2</v>
       </c>
     </row>
@@ -2145,13 +2255,13 @@
       <c r="B14" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="7">
         <v>0</v>
       </c>
     </row>
@@ -2159,13 +2269,13 @@
       <c r="B15" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="7">
         <v>0</v>
       </c>
     </row>
@@ -2173,13 +2283,13 @@
       <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="22">
         <v>12</v>
       </c>
     </row>
@@ -2187,561 +2297,561 @@
       <c r="B17" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="24">
         <v>0.2</v>
       </c>
-      <c r="F17" s="10"/>
+      <c r="F17" s="7"/>
     </row>
     <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="24">
         <v>0.2</v>
       </c>
-      <c r="F18" s="10"/>
+      <c r="F18" s="7"/>
     </row>
     <row r="19" ht="16" spans="2:6">
       <c r="B19" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="24">
         <v>0.2</v>
       </c>
-      <c r="F19" s="10"/>
+      <c r="F19" s="7"/>
     </row>
     <row r="20" spans="2:6">
       <c r="B20" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="24">
         <v>0.5</v>
       </c>
-      <c r="F20" s="10"/>
+      <c r="F20" s="7"/>
     </row>
     <row r="21" ht="16" spans="2:6">
       <c r="B21" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="24">
         <v>0.8</v>
       </c>
-      <c r="F21" s="10"/>
+      <c r="F21" s="7"/>
     </row>
     <row r="22" ht="16" spans="2:6">
       <c r="B22" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="9"/>
-      <c r="F22" s="10"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="7"/>
     </row>
     <row r="23" spans="2:6">
       <c r="B23" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E23" s="10">
-        <v>1</v>
-      </c>
-      <c r="F23" s="10"/>
+      <c r="E23" s="7">
+        <v>1</v>
+      </c>
+      <c r="F23" s="7"/>
     </row>
     <row r="24" spans="2:6">
       <c r="B24" t="s">
         <v>17</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E24" s="10">
-        <v>1</v>
-      </c>
-      <c r="F24" s="10"/>
+      <c r="E24" s="7">
+        <v>1</v>
+      </c>
+      <c r="F24" s="7"/>
     </row>
     <row r="25" ht="16" spans="2:6">
       <c r="B25" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E25" s="10">
-        <v>1</v>
-      </c>
-      <c r="F25" s="10"/>
+      <c r="E25" s="7">
+        <v>1</v>
+      </c>
+      <c r="F25" s="7"/>
     </row>
     <row r="26" spans="2:6">
       <c r="B26" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="17">
         <v>0.05</v>
       </c>
-      <c r="F26" s="10"/>
+      <c r="F26" s="7"/>
     </row>
     <row r="27" spans="2:6">
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D27" s="20" t="s">
+      <c r="D27" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="20">
+      <c r="E27" s="25">
         <v>2020</v>
       </c>
-      <c r="F27" s="10"/>
+      <c r="F27" s="7"/>
     </row>
     <row r="28" spans="2:6">
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="D28" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="E28" s="21">
+      <c r="E28" s="26">
         <v>2020</v>
       </c>
-      <c r="F28" s="10"/>
+      <c r="F28" s="7"/>
     </row>
     <row r="29" spans="2:6">
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
     </row>
     <row r="30" spans="2:6">
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
     </row>
     <row r="31" spans="2:6">
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
     </row>
     <row r="32" spans="2:6">
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
     </row>
     <row r="38" spans="3:5">
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
     </row>
     <row r="54" spans="3:11">
-      <c r="C54" s="22" t="s">
+      <c r="C54" s="27" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="56" spans="3:11">
-      <c r="D56" s="22"/>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="22"/>
-      <c r="I56" s="22"/>
-      <c r="J56" s="22"/>
-      <c r="K56" s="22"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="27"/>
+      <c r="G56" s="27"/>
+      <c r="H56" s="27"/>
+      <c r="I56" s="27"/>
+      <c r="J56" s="27"/>
+      <c r="K56" s="27"/>
     </row>
     <row r="57" spans="3:11">
-      <c r="C57" s="22" t="s">
+      <c r="C57" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="D57" s="22" t="s">
+      <c r="D57" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="E57" s="22" t="s">
+      <c r="E57" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="F57" s="22" t="s">
+      <c r="F57" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="G57" s="22" t="s">
+      <c r="G57" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="H57" s="22" t="s">
+      <c r="H57" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="I57" s="22" t="s">
+      <c r="I57" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="J57" s="22" t="s">
+      <c r="J57" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="K57" s="22" t="s">
+      <c r="K57" s="27" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="58" spans="3:11">
-      <c r="C58" s="22"/>
-      <c r="D58" s="22"/>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="22"/>
-      <c r="H58" s="22"/>
-      <c r="I58" s="22"/>
-      <c r="J58" s="22"/>
-      <c r="K58" s="22"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="27"/>
+      <c r="F58" s="27"/>
+      <c r="G58" s="27"/>
+      <c r="H58" s="27"/>
+      <c r="I58" s="27"/>
+      <c r="J58" s="27"/>
+      <c r="K58" s="27"/>
     </row>
     <row r="59" spans="3:11">
-      <c r="C59" s="22"/>
-      <c r="D59" s="22"/>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
-      <c r="K59" s="22"/>
+      <c r="C59" s="27"/>
+      <c r="D59" s="27"/>
+      <c r="E59" s="27"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="27"/>
+      <c r="H59" s="27"/>
+      <c r="I59" s="27"/>
+      <c r="J59" s="27"/>
+      <c r="K59" s="27"/>
     </row>
     <row r="60" spans="3:11">
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
-      <c r="K60" s="22"/>
+      <c r="C60" s="27"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="27"/>
+      <c r="F60" s="27"/>
+      <c r="G60" s="27"/>
+      <c r="H60" s="27"/>
+      <c r="I60" s="27"/>
+      <c r="J60" s="27"/>
+      <c r="K60" s="27"/>
     </row>
     <row r="61" spans="3:11">
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
-      <c r="G61" s="22"/>
-      <c r="H61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
-      <c r="K61" s="22"/>
+      <c r="C61" s="27"/>
+      <c r="D61" s="27"/>
+      <c r="E61" s="27"/>
+      <c r="F61" s="27"/>
+      <c r="G61" s="27"/>
+      <c r="H61" s="27"/>
+      <c r="I61" s="27"/>
+      <c r="J61" s="27"/>
+      <c r="K61" s="27"/>
     </row>
     <row r="62" spans="3:11">
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="22"/>
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
-      <c r="K62" s="22"/>
+      <c r="C62" s="27"/>
+      <c r="D62" s="27"/>
+      <c r="E62" s="27"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="27"/>
+      <c r="H62" s="27"/>
+      <c r="I62" s="27"/>
+      <c r="J62" s="27"/>
+      <c r="K62" s="27"/>
     </row>
     <row r="63" spans="3:11">
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="22"/>
-      <c r="H63" s="22"/>
-      <c r="I63" s="22"/>
-      <c r="J63" s="22"/>
-      <c r="K63" s="22"/>
+      <c r="C63" s="27"/>
+      <c r="D63" s="27"/>
+      <c r="E63" s="27"/>
+      <c r="F63" s="27"/>
+      <c r="G63" s="27"/>
+      <c r="H63" s="27"/>
+      <c r="I63" s="27"/>
+      <c r="J63" s="27"/>
+      <c r="K63" s="27"/>
     </row>
     <row r="64" spans="3:11">
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="22"/>
-      <c r="H64" s="22"/>
-      <c r="I64" s="22"/>
-      <c r="J64" s="22"/>
-      <c r="K64" s="22"/>
+      <c r="C64" s="27"/>
+      <c r="D64" s="27"/>
+      <c r="E64" s="27"/>
+      <c r="F64" s="27"/>
+      <c r="G64" s="27"/>
+      <c r="H64" s="27"/>
+      <c r="I64" s="27"/>
+      <c r="J64" s="27"/>
+      <c r="K64" s="27"/>
     </row>
     <row r="65" spans="3:11">
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="22"/>
-      <c r="G65" s="22"/>
-      <c r="H65" s="22"/>
-      <c r="I65" s="22"/>
-      <c r="J65" s="22"/>
-      <c r="K65" s="22"/>
+      <c r="C65" s="27"/>
+      <c r="D65" s="27"/>
+      <c r="E65" s="27"/>
+      <c r="F65" s="27"/>
+      <c r="G65" s="27"/>
+      <c r="H65" s="27"/>
+      <c r="I65" s="27"/>
+      <c r="J65" s="27"/>
+      <c r="K65" s="27"/>
     </row>
     <row r="66" spans="3:11">
-      <c r="C66" s="22"/>
-      <c r="D66" s="22"/>
-      <c r="E66" s="22"/>
-      <c r="F66" s="22"/>
-      <c r="G66" s="22"/>
-      <c r="H66" s="22"/>
-      <c r="I66" s="22"/>
-      <c r="J66" s="22"/>
-      <c r="K66" s="22"/>
+      <c r="C66" s="27"/>
+      <c r="D66" s="27"/>
+      <c r="E66" s="27"/>
+      <c r="F66" s="27"/>
+      <c r="G66" s="27"/>
+      <c r="H66" s="27"/>
+      <c r="I66" s="27"/>
+      <c r="J66" s="27"/>
+      <c r="K66" s="27"/>
     </row>
     <row r="67" spans="3:11">
-      <c r="C67" s="22"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="22"/>
-      <c r="F67" s="22"/>
-      <c r="G67" s="22"/>
-      <c r="H67" s="22"/>
-      <c r="I67" s="22"/>
-      <c r="J67" s="22"/>
-      <c r="K67" s="22"/>
+      <c r="C67" s="27"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="27"/>
+      <c r="F67" s="27"/>
+      <c r="G67" s="27"/>
+      <c r="H67" s="27"/>
+      <c r="I67" s="27"/>
+      <c r="J67" s="27"/>
+      <c r="K67" s="27"/>
     </row>
     <row r="68" spans="3:11">
-      <c r="C68" s="22"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="22"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="22"/>
-      <c r="I68" s="22"/>
-      <c r="J68" s="22"/>
-      <c r="K68" s="22"/>
+      <c r="C68" s="27"/>
+      <c r="D68" s="27"/>
+      <c r="E68" s="27"/>
+      <c r="F68" s="27"/>
+      <c r="G68" s="27"/>
+      <c r="H68" s="27"/>
+      <c r="I68" s="27"/>
+      <c r="J68" s="27"/>
+      <c r="K68" s="27"/>
     </row>
     <row r="69" spans="3:11">
-      <c r="C69" s="22"/>
-      <c r="D69" s="22"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="22"/>
-      <c r="I69" s="22"/>
-      <c r="J69" s="22"/>
-      <c r="K69" s="22"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="27"/>
+      <c r="G69" s="27"/>
+      <c r="H69" s="27"/>
+      <c r="I69" s="27"/>
+      <c r="J69" s="27"/>
+      <c r="K69" s="27"/>
     </row>
     <row r="70" spans="3:11">
-      <c r="C70" s="22"/>
-      <c r="D70" s="22"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
-      <c r="G70" s="22"/>
-      <c r="H70" s="22"/>
-      <c r="I70" s="22"/>
-      <c r="J70" s="22"/>
-      <c r="K70" s="22"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="27"/>
+      <c r="E70" s="27"/>
+      <c r="F70" s="27"/>
+      <c r="G70" s="27"/>
+      <c r="H70" s="27"/>
+      <c r="I70" s="27"/>
+      <c r="J70" s="27"/>
+      <c r="K70" s="27"/>
     </row>
     <row r="71" spans="3:11">
-      <c r="C71" s="22"/>
-      <c r="D71" s="22"/>
-      <c r="E71" s="22"/>
-      <c r="F71" s="22"/>
-      <c r="G71" s="22"/>
-      <c r="H71" s="22"/>
-      <c r="I71" s="22"/>
-      <c r="J71" s="22"/>
-      <c r="K71" s="22"/>
+      <c r="C71" s="27"/>
+      <c r="D71" s="27"/>
+      <c r="E71" s="27"/>
+      <c r="F71" s="27"/>
+      <c r="G71" s="27"/>
+      <c r="H71" s="27"/>
+      <c r="I71" s="27"/>
+      <c r="J71" s="27"/>
+      <c r="K71" s="27"/>
     </row>
     <row r="72" spans="3:11">
-      <c r="C72" s="22"/>
-      <c r="D72" s="22"/>
-      <c r="E72" s="22"/>
-      <c r="F72" s="22"/>
-      <c r="G72" s="22"/>
-      <c r="H72" s="22"/>
-      <c r="I72" s="22"/>
-      <c r="J72" s="22"/>
-      <c r="K72" s="22"/>
+      <c r="C72" s="27"/>
+      <c r="D72" s="27"/>
+      <c r="E72" s="27"/>
+      <c r="F72" s="27"/>
+      <c r="G72" s="27"/>
+      <c r="H72" s="27"/>
+      <c r="I72" s="27"/>
+      <c r="J72" s="27"/>
+      <c r="K72" s="27"/>
     </row>
     <row r="73" spans="3:11">
-      <c r="C73" s="22"/>
-      <c r="D73" s="22"/>
-      <c r="E73" s="22"/>
-      <c r="F73" s="22"/>
-      <c r="G73" s="22"/>
-      <c r="H73" s="22"/>
-      <c r="I73" s="22"/>
-      <c r="J73" s="22"/>
-      <c r="K73" s="22"/>
+      <c r="C73" s="27"/>
+      <c r="D73" s="27"/>
+      <c r="E73" s="27"/>
+      <c r="F73" s="27"/>
+      <c r="G73" s="27"/>
+      <c r="H73" s="27"/>
+      <c r="I73" s="27"/>
+      <c r="J73" s="27"/>
+      <c r="K73" s="27"/>
     </row>
     <row r="74" spans="3:11">
-      <c r="C74" s="22"/>
-      <c r="D74" s="22"/>
-      <c r="E74" s="22"/>
-      <c r="F74" s="22"/>
-      <c r="G74" s="22"/>
-      <c r="H74" s="22"/>
-      <c r="I74" s="22"/>
-      <c r="J74" s="22"/>
-      <c r="K74" s="22"/>
+      <c r="C74" s="27"/>
+      <c r="D74" s="27"/>
+      <c r="E74" s="27"/>
+      <c r="F74" s="27"/>
+      <c r="G74" s="27"/>
+      <c r="H74" s="27"/>
+      <c r="I74" s="27"/>
+      <c r="J74" s="27"/>
+      <c r="K74" s="27"/>
     </row>
     <row r="75" spans="3:11">
-      <c r="C75" s="22"/>
-      <c r="D75" s="22"/>
-      <c r="E75" s="22"/>
-      <c r="F75" s="22"/>
-      <c r="G75" s="22"/>
-      <c r="H75" s="22"/>
-      <c r="I75" s="22"/>
-      <c r="J75" s="22"/>
-      <c r="K75" s="22"/>
+      <c r="C75" s="27"/>
+      <c r="D75" s="27"/>
+      <c r="E75" s="27"/>
+      <c r="F75" s="27"/>
+      <c r="G75" s="27"/>
+      <c r="H75" s="27"/>
+      <c r="I75" s="27"/>
+      <c r="J75" s="27"/>
+      <c r="K75" s="27"/>
     </row>
     <row r="76" spans="3:11">
-      <c r="C76" s="22"/>
-      <c r="D76" s="22"/>
-      <c r="E76" s="22"/>
-      <c r="F76" s="22"/>
-      <c r="G76" s="22"/>
-      <c r="H76" s="22"/>
-      <c r="I76" s="22"/>
-      <c r="J76" s="22"/>
-      <c r="K76" s="22"/>
+      <c r="C76" s="27"/>
+      <c r="D76" s="27"/>
+      <c r="E76" s="27"/>
+      <c r="F76" s="27"/>
+      <c r="G76" s="27"/>
+      <c r="H76" s="27"/>
+      <c r="I76" s="27"/>
+      <c r="J76" s="27"/>
+      <c r="K76" s="27"/>
     </row>
     <row r="77" spans="3:11">
-      <c r="C77" s="22"/>
-      <c r="D77" s="22"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="22"/>
-      <c r="G77" s="22"/>
-      <c r="H77" s="22"/>
-      <c r="I77" s="22"/>
-      <c r="J77" s="22"/>
-      <c r="K77" s="22"/>
+      <c r="C77" s="27"/>
+      <c r="D77" s="27"/>
+      <c r="E77" s="27"/>
+      <c r="F77" s="27"/>
+      <c r="G77" s="27"/>
+      <c r="H77" s="27"/>
+      <c r="I77" s="27"/>
+      <c r="J77" s="27"/>
+      <c r="K77" s="27"/>
     </row>
     <row r="78" spans="3:11">
-      <c r="C78" s="22"/>
-      <c r="D78" s="22"/>
-      <c r="E78" s="22"/>
-      <c r="F78" s="22"/>
-      <c r="G78" s="22"/>
-      <c r="H78" s="22"/>
-      <c r="I78" s="22"/>
-      <c r="J78" s="22"/>
-      <c r="K78" s="22"/>
+      <c r="C78" s="27"/>
+      <c r="D78" s="27"/>
+      <c r="E78" s="27"/>
+      <c r="F78" s="27"/>
+      <c r="G78" s="27"/>
+      <c r="H78" s="27"/>
+      <c r="I78" s="27"/>
+      <c r="J78" s="27"/>
+      <c r="K78" s="27"/>
     </row>
     <row r="79" spans="3:11">
-      <c r="C79" s="22"/>
-      <c r="D79" s="22"/>
-      <c r="E79" s="22"/>
-      <c r="F79" s="22"/>
-      <c r="G79" s="22"/>
-      <c r="H79" s="22"/>
-      <c r="I79" s="22"/>
-      <c r="J79" s="22"/>
-      <c r="K79" s="22"/>
+      <c r="C79" s="27"/>
+      <c r="D79" s="27"/>
+      <c r="E79" s="27"/>
+      <c r="F79" s="27"/>
+      <c r="G79" s="27"/>
+      <c r="H79" s="27"/>
+      <c r="I79" s="27"/>
+      <c r="J79" s="27"/>
+      <c r="K79" s="27"/>
     </row>
     <row r="80" spans="3:11">
-      <c r="C80" s="22"/>
-      <c r="D80" s="22"/>
-      <c r="E80" s="22"/>
-      <c r="F80" s="22"/>
-      <c r="G80" s="22"/>
-      <c r="H80" s="22"/>
-      <c r="I80" s="22"/>
-      <c r="J80" s="22"/>
-      <c r="K80" s="22"/>
+      <c r="C80" s="27"/>
+      <c r="D80" s="27"/>
+      <c r="E80" s="27"/>
+      <c r="F80" s="27"/>
+      <c r="G80" s="27"/>
+      <c r="H80" s="27"/>
+      <c r="I80" s="27"/>
+      <c r="J80" s="27"/>
+      <c r="K80" s="27"/>
     </row>
     <row r="81" spans="3:11">
-      <c r="C81" s="22"/>
-      <c r="D81" s="22"/>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
-      <c r="G81" s="22"/>
-      <c r="H81" s="22"/>
-      <c r="I81" s="22"/>
-      <c r="J81" s="22"/>
-      <c r="K81" s="22"/>
+      <c r="C81" s="27"/>
+      <c r="D81" s="27"/>
+      <c r="E81" s="27"/>
+      <c r="F81" s="27"/>
+      <c r="G81" s="27"/>
+      <c r="H81" s="27"/>
+      <c r="I81" s="27"/>
+      <c r="J81" s="27"/>
+      <c r="K81" s="27"/>
     </row>
     <row r="82" spans="3:11">
-      <c r="C82" s="22"/>
-      <c r="D82" s="22"/>
-      <c r="E82" s="22"/>
-      <c r="F82" s="22"/>
-      <c r="G82" s="22"/>
-      <c r="H82" s="22"/>
-      <c r="I82" s="22"/>
-      <c r="J82" s="22"/>
-      <c r="K82" s="22"/>
+      <c r="C82" s="27"/>
+      <c r="D82" s="27"/>
+      <c r="E82" s="27"/>
+      <c r="F82" s="27"/>
+      <c r="G82" s="27"/>
+      <c r="H82" s="27"/>
+      <c r="I82" s="27"/>
+      <c r="J82" s="27"/>
+      <c r="K82" s="27"/>
     </row>
     <row r="83" spans="3:11">
-      <c r="C83" s="22"/>
-      <c r="D83" s="22"/>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
-      <c r="G83" s="22"/>
-      <c r="H83" s="22"/>
-      <c r="I83" s="22"/>
-      <c r="J83" s="22"/>
-      <c r="K83" s="22"/>
+      <c r="C83" s="27"/>
+      <c r="D83" s="27"/>
+      <c r="E83" s="27"/>
+      <c r="F83" s="27"/>
+      <c r="G83" s="27"/>
+      <c r="H83" s="27"/>
+      <c r="I83" s="27"/>
+      <c r="J83" s="27"/>
+      <c r="K83" s="27"/>
     </row>
     <row r="84" spans="3:11">
-      <c r="C84" s="22" t="s">
+      <c r="C84" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="D84" s="22">
-        <v>1</v>
-      </c>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
-      <c r="G84" s="22"/>
-      <c r="H84" s="22"/>
-      <c r="I84" s="22"/>
-      <c r="J84" s="22"/>
-      <c r="K84" s="22"/>
+      <c r="D84" s="27">
+        <v>1</v>
+      </c>
+      <c r="E84" s="27"/>
+      <c r="F84" s="27"/>
+      <c r="G84" s="27"/>
+      <c r="H84" s="27"/>
+      <c r="I84" s="27"/>
+      <c r="J84" s="27"/>
+      <c r="K84" s="27"/>
     </row>
     <row r="85" spans="3:11">
-      <c r="C85" s="22"/>
-      <c r="D85" s="22"/>
-      <c r="E85" s="22"/>
-      <c r="F85" s="22"/>
-      <c r="G85" s="22"/>
-      <c r="H85" s="22"/>
-      <c r="I85" s="22"/>
-      <c r="J85" s="22"/>
-      <c r="K85" s="22"/>
+      <c r="C85" s="27"/>
+      <c r="D85" s="27"/>
+      <c r="E85" s="27"/>
+      <c r="F85" s="27"/>
+      <c r="G85" s="27"/>
+      <c r="H85" s="27"/>
+      <c r="I85" s="27"/>
+      <c r="J85" s="27"/>
+      <c r="K85" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2753,7 +2863,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B2:N52"/>
+  <dimension ref="B2:N54"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
   <cols>
     <col min="4" max="4" width="27.1636363636364" customWidth="1"/>
@@ -2782,255 +2892,255 @@
       </c>
     </row>
     <row r="8" spans="2:14">
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="M8" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="N8" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" spans="2:14">
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J9">
         <v>1</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="5">
         <v>1.25</v>
       </c>
       <c r="L9">
         <v>0.05</v>
       </c>
-      <c r="M9" s="2">
-        <v>1</v>
-      </c>
-      <c r="N9" s="2"/>
+      <c r="M9" s="5">
+        <v>1</v>
+      </c>
+      <c r="N9" s="5"/>
     </row>
     <row r="10" spans="2:14">
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J10">
         <v>1</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="5">
         <v>1.11</v>
       </c>
       <c r="L10">
         <v>0.05</v>
       </c>
-      <c r="M10" s="2">
-        <v>1</v>
-      </c>
-      <c r="N10" s="2"/>
+      <c r="M10" s="5">
+        <v>1</v>
+      </c>
+      <c r="N10" s="5"/>
     </row>
     <row r="11" spans="2:14">
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J11">
         <v>1</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="5">
         <v>1.15</v>
       </c>
       <c r="L11">
         <v>0.08</v>
       </c>
-      <c r="M11" s="2">
-        <v>1</v>
-      </c>
-      <c r="N11" s="2"/>
+      <c r="M11" s="5">
+        <v>1</v>
+      </c>
+      <c r="N11" s="5"/>
     </row>
     <row r="12" ht="16" spans="2:14">
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J12">
         <v>1</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="5">
         <v>1.12</v>
       </c>
       <c r="L12">
         <v>0.03</v>
       </c>
-      <c r="M12" s="2">
-        <v>1</v>
-      </c>
-      <c r="N12" s="2"/>
+      <c r="M12" s="5">
+        <v>1</v>
+      </c>
+      <c r="N12" s="5"/>
     </row>
     <row r="13" spans="2:14">
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J13">
         <v>1</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="5">
         <v>1.2</v>
       </c>
       <c r="L13">
         <v>0.1</v>
       </c>
-      <c r="M13" s="2">
-        <v>1</v>
-      </c>
-      <c r="N13" s="2"/>
+      <c r="M13" s="5">
+        <v>1</v>
+      </c>
+      <c r="N13" s="5"/>
     </row>
     <row r="14" spans="2:14">
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J14">
         <v>1</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="5">
         <v>1.06</v>
       </c>
       <c r="L14">
         <v>0.15</v>
       </c>
-      <c r="M14" s="2">
-        <v>1</v>
-      </c>
-      <c r="N14" s="2"/>
+      <c r="M14" s="5">
+        <v>1</v>
+      </c>
+      <c r="N14" s="5"/>
     </row>
     <row r="15" spans="2:14">
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J15">
         <v>1</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="5">
         <v>1.06</v>
       </c>
       <c r="L15">
         <v>0.3</v>
       </c>
-      <c r="M15" s="2">
-        <v>1</v>
-      </c>
-      <c r="N15" s="2"/>
+      <c r="M15" s="5">
+        <v>1</v>
+      </c>
+      <c r="N15" s="5"/>
     </row>
     <row r="16" ht="16" spans="2:14">
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="6" t="s">
         <v>86</v>
       </c>
       <c r="G16" t="str">
@@ -3041,7 +3151,7 @@
         <f>H15</f>
         <v>2025, 2150</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J16">
@@ -3062,10 +3172,10 @@
       </c>
     </row>
     <row r="17" ht="16" spans="4:14">
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="6" t="s">
         <v>88</v>
       </c>
       <c r="G17" t="str">
@@ -3076,7 +3186,7 @@
         <f t="shared" si="1"/>
         <v>2025, 2150</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="I17" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J17">
@@ -3097,10 +3207,10 @@
       </c>
     </row>
     <row r="18" ht="16" spans="4:14">
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="6" t="s">
         <v>90</v>
       </c>
       <c r="G18" t="str">
@@ -3111,7 +3221,7 @@
         <f>H17</f>
         <v>2025, 2150</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J18">
@@ -3127,309 +3237,1015 @@
         <v>1</v>
       </c>
     </row>
+    <row r="27" spans="4:14">
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+    </row>
     <row r="28" spans="4:14">
-      <c r="H28" t="s">
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7" t="s">
         <v>59</v>
       </c>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
     </row>
     <row r="29" spans="4:14">
-      <c r="D29" t="s">
+      <c r="D29" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="I29" t="s">
+      <c r="I29" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="K29" t="s">
+      <c r="K29" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="L29" t="s">
+      <c r="L29" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="M29" t="s">
+      <c r="M29" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="N29" t="s">
+      <c r="N29" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="30" ht="16" spans="4:14">
-      <c r="D30" t="s">
+      <c r="D30" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="E30" s="7"/>
+      <c r="F30" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H30" t="s">
+      <c r="H30" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I30" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J30">
-        <v>1</v>
-      </c>
-      <c r="K30">
-        <v>1</v>
-      </c>
-      <c r="L30">
+      <c r="J30" s="7">
+        <v>1</v>
+      </c>
+      <c r="K30" s="7">
+        <v>1</v>
+      </c>
+      <c r="L30" s="7">
         <v>0.01</v>
       </c>
-      <c r="M30">
-        <v>1</v>
-      </c>
+      <c r="M30" s="7">
+        <v>1</v>
+      </c>
+      <c r="N30" s="7"/>
     </row>
     <row r="31" ht="16" spans="4:14">
-      <c r="D31" t="s">
+      <c r="D31" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="E31" s="7"/>
+      <c r="F31" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J31">
-        <v>1</v>
-      </c>
-      <c r="K31">
-        <v>1</v>
-      </c>
-      <c r="L31">
+      <c r="J31" s="7">
+        <v>1</v>
+      </c>
+      <c r="K31" s="7">
+        <v>1</v>
+      </c>
+      <c r="L31" s="7">
         <f t="shared" ref="L31:L36" si="2">L30</f>
         <v>0.01</v>
       </c>
-      <c r="M31">
-        <v>1</v>
-      </c>
+      <c r="M31" s="7">
+        <v>1</v>
+      </c>
+      <c r="N31" s="7"/>
     </row>
     <row r="32" ht="16" spans="4:14">
-      <c r="D32" t="s">
+      <c r="D32" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="E32" s="7"/>
+      <c r="F32" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H32" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J32">
-        <v>1</v>
-      </c>
-      <c r="K32">
-        <v>1</v>
-      </c>
-      <c r="L32">
+      <c r="J32" s="7">
+        <v>1</v>
+      </c>
+      <c r="K32" s="7">
+        <v>1</v>
+      </c>
+      <c r="L32" s="7">
         <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="M32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" ht="16" spans="4:13">
-      <c r="D33" t="s">
+      <c r="M32" s="7">
+        <v>1</v>
+      </c>
+      <c r="N32" s="7"/>
+    </row>
+    <row r="33" ht="16" spans="4:14">
+      <c r="D33" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="E33" s="7"/>
+      <c r="F33" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H33" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J33">
-        <v>1</v>
-      </c>
-      <c r="K33">
+      <c r="J33" s="7">
+        <v>1</v>
+      </c>
+      <c r="K33" s="7">
         <f>K32</f>
         <v>1</v>
       </c>
-      <c r="L33">
+      <c r="L33" s="7">
         <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="M33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" ht="16" spans="4:13">
-      <c r="D34" t="s">
+      <c r="M33" s="7">
+        <v>1</v>
+      </c>
+      <c r="N33" s="7"/>
+    </row>
+    <row r="34" ht="16" spans="4:14">
+      <c r="D34" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="E34" s="7"/>
+      <c r="F34" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H34" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I34" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J34">
-        <v>1</v>
-      </c>
-      <c r="K34">
+      <c r="J34" s="7">
+        <v>1</v>
+      </c>
+      <c r="K34" s="7">
         <f>K33</f>
         <v>1</v>
       </c>
-      <c r="L34">
+      <c r="L34" s="7">
         <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="M34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" ht="16" spans="4:13">
-      <c r="D35" t="s">
+      <c r="M34" s="7">
+        <v>1</v>
+      </c>
+      <c r="N34" s="7"/>
+    </row>
+    <row r="35" ht="16" spans="4:14">
+      <c r="D35" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="E35" s="7"/>
+      <c r="F35" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H35" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J35">
-        <v>1</v>
-      </c>
-      <c r="K35">
-        <f>K34</f>
-        <v>1</v>
-      </c>
-      <c r="L35">
+      <c r="J35" s="7">
+        <v>1</v>
+      </c>
+      <c r="K35" s="7">
+        <f t="shared" ref="K35:K43" si="3">K34</f>
+        <v>1</v>
+      </c>
+      <c r="L35" s="7">
         <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="M35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" ht="16" spans="4:13">
-      <c r="D36" t="s">
+      <c r="M35" s="7">
+        <v>1</v>
+      </c>
+      <c r="N35" s="7"/>
+    </row>
+    <row r="36" ht="16" spans="4:14">
+      <c r="D36" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="E36" s="7"/>
+      <c r="F36" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H36" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J36">
-        <v>1</v>
-      </c>
-      <c r="K36">
-        <f>K35</f>
-        <v>1</v>
-      </c>
-      <c r="L36">
+      <c r="J36" s="7">
+        <v>1</v>
+      </c>
+      <c r="K36" s="7">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="L36" s="7">
         <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="M36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="4:13">
-      <c r="F37" s="5"/>
-    </row>
-    <row r="38" spans="4:13">
-      <c r="F38" s="5"/>
-    </row>
-    <row r="39" spans="4:13">
-      <c r="F39" s="5"/>
-    </row>
-    <row r="40" spans="4:13">
-      <c r="F40" s="5"/>
-    </row>
-    <row r="41" spans="4:13">
-      <c r="F41" s="5"/>
-    </row>
-    <row r="42" spans="4:13">
-      <c r="F42" s="5"/>
-    </row>
-    <row r="43" spans="4:13">
-      <c r="F43" s="5"/>
-    </row>
-    <row r="44" spans="4:13">
-      <c r="F44" s="5"/>
-    </row>
-    <row r="45" spans="4:13">
-      <c r="F45" s="5"/>
-    </row>
-    <row r="46" spans="4:13">
-      <c r="F46" s="5"/>
-    </row>
-    <row r="47" spans="4:13">
-      <c r="F47" s="5"/>
-    </row>
-    <row r="48" spans="4:13">
-      <c r="F48" s="5"/>
-    </row>
-    <row r="49" spans="6:6">
-      <c r="F49" s="5"/>
-    </row>
-    <row r="50" spans="6:6">
-      <c r="F50" s="6"/>
-    </row>
-    <row r="51" spans="6:6">
-      <c r="F51" s="7"/>
-    </row>
-    <row r="52" spans="6:6">
-      <c r="F52" s="7"/>
+      <c r="M36" s="7">
+        <v>1</v>
+      </c>
+      <c r="N36" s="7"/>
+    </row>
+    <row r="37" ht="16" spans="4:14">
+      <c r="D37" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E37" s="10"/>
+      <c r="F37" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J37" s="10">
+        <v>1</v>
+      </c>
+      <c r="K37" s="10">
+        <v>1</v>
+      </c>
+      <c r="L37" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="M37" s="10">
+        <v>1</v>
+      </c>
+      <c r="N37" s="7"/>
+    </row>
+    <row r="38" ht="16" spans="4:14">
+      <c r="D38" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E38" s="10"/>
+      <c r="F38" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I38" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J38" s="10">
+        <v>1</v>
+      </c>
+      <c r="K38" s="10">
+        <v>1</v>
+      </c>
+      <c r="L38" s="10">
+        <f t="shared" ref="L38:L43" si="4">L37</f>
+        <v>0.01</v>
+      </c>
+      <c r="M38" s="10">
+        <v>1</v>
+      </c>
+      <c r="N38" s="7"/>
+    </row>
+    <row r="39" ht="16" spans="4:14">
+      <c r="D39" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E39" s="10"/>
+      <c r="F39" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J39" s="10">
+        <v>1</v>
+      </c>
+      <c r="K39" s="10">
+        <v>1</v>
+      </c>
+      <c r="L39" s="10">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="M39" s="10">
+        <v>1</v>
+      </c>
+      <c r="N39" s="7"/>
+    </row>
+    <row r="40" ht="16" spans="4:14">
+      <c r="D40" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E40" s="10"/>
+      <c r="F40" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I40" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J40" s="10">
+        <v>1</v>
+      </c>
+      <c r="K40" s="10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="L40" s="10">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="M40" s="10">
+        <v>1</v>
+      </c>
+      <c r="N40" s="7"/>
+    </row>
+    <row r="41" ht="16" spans="4:14">
+      <c r="D41" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="10"/>
+      <c r="F41" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J41" s="10">
+        <v>1</v>
+      </c>
+      <c r="K41" s="10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="L41" s="10">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="M41" s="10">
+        <v>1</v>
+      </c>
+      <c r="N41" s="7"/>
+    </row>
+    <row r="42" ht="16" spans="4:14">
+      <c r="D42" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E42" s="10"/>
+      <c r="F42" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="G42" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I42" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J42" s="10">
+        <v>1</v>
+      </c>
+      <c r="K42" s="10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="L42" s="10">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="M42" s="10">
+        <v>1</v>
+      </c>
+      <c r="N42" s="7"/>
+    </row>
+    <row r="43" ht="16" spans="4:14">
+      <c r="D43" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E43" s="10"/>
+      <c r="F43" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="J43" s="10">
+        <v>1</v>
+      </c>
+      <c r="K43" s="10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="L43" s="10">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="M43" s="10">
+        <v>1</v>
+      </c>
+      <c r="N43" s="7"/>
+    </row>
+    <row r="44" spans="4:14">
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="10"/>
+      <c r="N44" s="7"/>
+    </row>
+    <row r="45" spans="4:14">
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10"/>
+      <c r="L45" s="10"/>
+      <c r="M45" s="10"/>
+      <c r="N45" s="7"/>
+    </row>
+    <row r="46" spans="4:14">
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="7"/>
+      <c r="K46" s="7"/>
+      <c r="L46" s="7"/>
+      <c r="M46" s="7"/>
+      <c r="N46" s="7"/>
+    </row>
+    <row r="47" spans="4:14">
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="7"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="7"/>
+      <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
+    </row>
+    <row r="48" spans="4:14">
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="7"/>
+      <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
+    </row>
+    <row r="49" spans="4:14">
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
+      <c r="N49" s="7"/>
+    </row>
+    <row r="50" spans="4:14">
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+    </row>
+    <row r="51" spans="4:14">
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="7"/>
+      <c r="M51" s="7"/>
+      <c r="N51" s="7"/>
+    </row>
+    <row r="52" spans="4:14">
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
+      <c r="J52" s="7"/>
+      <c r="K52" s="7"/>
+      <c r="L52" s="7"/>
+      <c r="M52" s="7"/>
+      <c r="N52" s="7"/>
+    </row>
+    <row r="53" spans="4:14">
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="7"/>
+      <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
+      <c r="N53" s="7"/>
+    </row>
+    <row r="54" spans="4:14">
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+      <c r="K54" s="7"/>
+      <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
+      <c r="N54" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="E13:U33"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="9" max="9" width="43.7272727272727" customWidth="1"/>
+    <col min="12" max="12" width="10.2727272727273" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="13" spans="5:21">
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
+      <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
+      <c r="T13" s="1"/>
+      <c r="U13" s="1"/>
+    </row>
+    <row r="14" spans="5:21">
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
+    </row>
+    <row r="15" spans="5:21">
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+    </row>
+    <row r="16" spans="5:21">
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+    </row>
+    <row r="17" spans="5:21">
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="1"/>
+      <c r="U17" s="1"/>
+    </row>
+    <row r="18" spans="5:21">
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="1"/>
+      <c r="U18" s="1"/>
+    </row>
+    <row r="19" spans="5:21">
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="1"/>
+    </row>
+    <row r="20" spans="5:21">
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="1"/>
+    </row>
+    <row r="21" spans="5:21">
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="1"/>
+      <c r="U21" s="1"/>
+    </row>
+    <row r="22" spans="5:21">
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="1"/>
+      <c r="U22" s="1"/>
+    </row>
+    <row r="23" spans="5:21">
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+    </row>
+    <row r="24" spans="5:21">
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+    </row>
+    <row r="26" spans="5:21">
+      <c r="F26" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="5:21">
+      <c r="L29" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" ht="15.25" spans="5:21">
+      <c r="F30" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" t="s">
+        <v>48</v>
+      </c>
+      <c r="I30" t="s">
+        <v>124</v>
+      </c>
+      <c r="J30" t="s">
+        <v>33</v>
+      </c>
+      <c r="K30" t="s">
+        <v>125</v>
+      </c>
+      <c r="L30" t="s">
+        <v>1</v>
+      </c>
+      <c r="M30" t="s">
+        <v>126</v>
+      </c>
+      <c r="N30" t="s">
+        <v>127</v>
+      </c>
+      <c r="O30" t="s">
+        <v>128</v>
+      </c>
+      <c r="P30" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" ht="16" spans="5:21">
+      <c r="F31" t="s">
+        <v>130</v>
+      </c>
+      <c r="G31" t="s">
+        <v>131</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I31" t="s">
+        <v>133</v>
+      </c>
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+      <c r="K31" t="s">
+        <v>17</v>
+      </c>
+      <c r="M31">
+        <v>-0.25</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="32" ht="15.25" spans="5:21">
+      <c r="K32" t="s">
+        <v>135</v>
+      </c>
+      <c r="N32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="9:13">
+      <c r="I33" t="s">
+        <v>136</v>
+      </c>
+      <c r="J33" t="s">
+        <v>17</v>
+      </c>
+      <c r="K33" t="s">
+        <v>17</v>
+      </c>
+      <c r="M33">
+        <v>-0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
claude on EV increase
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_zAK_fixes.xlsx
+++ b/SuppXLS/Scen_zAK_fixes.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Growth_rate" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="util_limit" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Elc_limit" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="EV_share" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" name="IQ_FWD_Q" vbProcedure="false">501</definedName>
@@ -238,7 +239,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="285">
   <si>
     <t xml:space="preserve">~TFM_UPD</t>
   </si>
@@ -972,7 +973,7 @@
     <t xml:space="preserve">*~UC_Sets: R_E: AllRegions</t>
   </si>
   <si>
-    <t xml:space="preserve">*~UC_T: UC_RHSRT  (TEST: EV calibration disabled)</t>
+    <t xml:space="preserve">*~UC_T: UC_RHSRT  (2026-10-29: replaced by EV_share sheet)</t>
   </si>
   <si>
     <t xml:space="preserve">UCE_EVBattCalib</t>
@@ -982,6 +983,117 @@
   </si>
   <si>
     <t xml:space="preserve">EV battery stock (GWh) &lt;= calibrated 2020/2025 values; no bound after 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV share of new vehicles, 2020 &amp; 2025 periods: IEA GEVO 2026 historical sales share (sales-weighted by model region), upper bound = 1.25 x share + 1pp (2020) / + 2pp (2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constraint per region &amp; period: sum NCAP(EV) &lt;= u x sum NCAP(all of mode). EV = BEV (elc) + PHEV (pih). Coefficients: EV rows = 1-u, non-EV rows = -u. u = upper bound share shown in the matching table at right/below (fraction).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~UC_T: UC_NCAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCE_EVshareHist_car</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_car_elc*,Trd_car_*-pih*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cars EV share of new vehicles &lt;= u (EV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_car_*,-Trd_car_elc*,-Trd_car_*-pih*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cars EV share of new vehicles &lt;= u (nonEV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCE_EVshareHist_lcv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_lcv_elc*,Trd_lcv_*-pih*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vans EV share of new vehicles &lt;= u (EV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_lcv_*,-Trd_lcv_elc*,-Trd_lcv_*-pih*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vans EV share of new vehicles &lt;= u (nonEV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCE_EVshareHist_bus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_bus_elc*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buses EV share of new vehicles &lt;= u (EV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_bus_*,-Trd_bus_elc*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buses EV share of new vehicles &lt;= u (nonEV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCE_EVshareHist_hdt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_hdt_elc*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trucks EV share of new vehicles &lt;= u (EV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_hdt_*,-Trd_hdt_elc*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trucks EV share of new vehicles &lt;= u (nonEV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCE_EVshareHist_2w3w</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_2w_elc*,Trd_3w_elc*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 and 3 wheelers EV share of new vehicles &lt;= u (EV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trd_2w_*,Trd_3w_*,-Trd_2w_elc*,-Trd_3w_elc*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 and 3 wheelers EV share of new vehicles &lt;= u (nonEV row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* Upper-bound EV share of new vehicles (%), for reference only (comment rows, not read by VEDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Cars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Vans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Buses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Trucks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*2 and 3 wheelers</t>
   </si>
 </sst>
 </file>
@@ -993,7 +1105,7 @@
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1103,6 +1215,13 @@
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -1264,7 +1383,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1430,6 +1549,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="11" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1890,6 +2013,3981 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:AQ42"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="42" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="0" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="0" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="I7" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="J7" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="K7" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="L7" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="M7" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="N7" s="0" t="s">
+        <v>210</v>
+      </c>
+      <c r="O7" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="P7" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q7" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="R7" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="S7" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="T7" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="U7" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="V7" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="W7" s="0" t="s">
+        <v>219</v>
+      </c>
+      <c r="X7" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="Y7" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="Z7" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="AA7" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="AB7" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="AC7" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="AD7" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="AE7" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="AF7" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="AG7" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="AH7" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="AI7" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="AJ7" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="AK7" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="AL7" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="AM7" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="AN7" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="AO7" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="AP7" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="AQ7" s="0" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <v>0.9896</v>
+      </c>
+      <c r="J8" s="0" t="n">
+        <v>0.9896</v>
+      </c>
+      <c r="K8" s="0" t="n">
+        <v>0.9778</v>
+      </c>
+      <c r="L8" s="0" t="n">
+        <v>0.8712</v>
+      </c>
+      <c r="M8" s="0" t="n">
+        <v>0.9702</v>
+      </c>
+      <c r="N8" s="0" t="n">
+        <v>0.7785</v>
+      </c>
+      <c r="O8" s="0" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="P8" s="0" t="n">
+        <v>0.9187</v>
+      </c>
+      <c r="Q8" s="0" t="n">
+        <v>0.9573</v>
+      </c>
+      <c r="R8" s="0" t="n">
+        <v>0.9594</v>
+      </c>
+      <c r="S8" s="0" t="n">
+        <v>0.8525</v>
+      </c>
+      <c r="T8" s="0" t="n">
+        <v>0.815</v>
+      </c>
+      <c r="U8" s="0" t="n">
+        <v>0.9579</v>
+      </c>
+      <c r="V8" s="0" t="n">
+        <v>0.941</v>
+      </c>
+      <c r="W8" s="0" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="X8" s="0" t="n">
+        <v>0.9885</v>
+      </c>
+      <c r="Y8" s="0" t="n">
+        <v>0.8975</v>
+      </c>
+      <c r="Z8" s="0" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AA8" s="0" t="n">
+        <v>0.9804</v>
+      </c>
+      <c r="AB8" s="0" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="AC8" s="0" t="n">
+        <v>0.9673</v>
+      </c>
+      <c r="AD8" s="0" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="AE8" s="0" t="n">
+        <v>0.0525</v>
+      </c>
+      <c r="AF8" s="0" t="n">
+        <v>0.9663</v>
+      </c>
+      <c r="AG8" s="0" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AH8" s="0" t="n">
+        <v>0.9888</v>
+      </c>
+      <c r="AI8" s="0" t="n">
+        <v>0.9889</v>
+      </c>
+      <c r="AJ8" s="0" t="n">
+        <v>0.9888</v>
+      </c>
+      <c r="AK8" s="0" t="n">
+        <v>0.9188</v>
+      </c>
+      <c r="AL8" s="0" t="n">
+        <v>0.6863</v>
+      </c>
+      <c r="AM8" s="0" t="n">
+        <v>0.815</v>
+      </c>
+      <c r="AN8" s="0" t="n">
+        <v>0.9874</v>
+      </c>
+      <c r="AO8" s="0" t="n">
+        <v>0.8525</v>
+      </c>
+      <c r="AP8" s="0" t="n">
+        <v>0.9868</v>
+      </c>
+      <c r="AQ8" s="0" t="n">
+        <v>0.9868</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="I9" s="0" t="n">
+        <v>-0.0104</v>
+      </c>
+      <c r="J9" s="0" t="n">
+        <v>-0.0104</v>
+      </c>
+      <c r="K9" s="0" t="n">
+        <v>-0.0223</v>
+      </c>
+      <c r="L9" s="0" t="n">
+        <v>-0.1288</v>
+      </c>
+      <c r="M9" s="0" t="n">
+        <v>-0.0298</v>
+      </c>
+      <c r="N9" s="0" t="n">
+        <v>-0.2215</v>
+      </c>
+      <c r="O9" s="0" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="P9" s="0" t="n">
+        <v>-0.0813</v>
+      </c>
+      <c r="Q9" s="0" t="n">
+        <v>-0.0427</v>
+      </c>
+      <c r="R9" s="0" t="n">
+        <v>-0.0406</v>
+      </c>
+      <c r="S9" s="0" t="n">
+        <v>-0.1475</v>
+      </c>
+      <c r="T9" s="0" t="n">
+        <v>-0.185</v>
+      </c>
+      <c r="U9" s="0" t="n">
+        <v>-0.0421</v>
+      </c>
+      <c r="V9" s="0" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="W9" s="0" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="X9" s="0" t="n">
+        <v>-0.0115</v>
+      </c>
+      <c r="Y9" s="0" t="n">
+        <v>-0.1025</v>
+      </c>
+      <c r="Z9" s="0" t="n">
+        <v>-0.0625</v>
+      </c>
+      <c r="AA9" s="0" t="n">
+        <v>-0.0196</v>
+      </c>
+      <c r="AB9" s="0" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="AC9" s="0" t="n">
+        <v>-0.0327</v>
+      </c>
+      <c r="AD9" s="0" t="n">
+        <v>-0.0395</v>
+      </c>
+      <c r="AE9" s="0" t="n">
+        <v>-0.9475</v>
+      </c>
+      <c r="AF9" s="0" t="n">
+        <v>-0.0338</v>
+      </c>
+      <c r="AG9" s="0" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="AH9" s="0" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="AI9" s="0" t="n">
+        <v>-0.0111</v>
+      </c>
+      <c r="AJ9" s="0" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="AK9" s="0" t="n">
+        <v>-0.0812</v>
+      </c>
+      <c r="AL9" s="0" t="n">
+        <v>-0.3137</v>
+      </c>
+      <c r="AM9" s="0" t="n">
+        <v>-0.185</v>
+      </c>
+      <c r="AN9" s="0" t="n">
+        <v>-0.0126</v>
+      </c>
+      <c r="AO9" s="0" t="n">
+        <v>-0.1475</v>
+      </c>
+      <c r="AP9" s="0" t="n">
+        <v>-0.0132</v>
+      </c>
+      <c r="AQ9" s="0" t="n">
+        <v>-0.0132</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <v>0.9675</v>
+      </c>
+      <c r="J10" s="0" t="n">
+        <v>0.9675</v>
+      </c>
+      <c r="K10" s="0" t="n">
+        <v>0.7925</v>
+      </c>
+      <c r="L10" s="0" t="n">
+        <v>0.5925</v>
+      </c>
+      <c r="M10" s="0" t="n">
+        <v>0.7535</v>
+      </c>
+      <c r="N10" s="0" t="n">
+        <v>0.3554</v>
+      </c>
+      <c r="O10" s="0" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="P10" s="0" t="n">
+        <v>0.3175</v>
+      </c>
+      <c r="Q10" s="0" t="n">
+        <v>0.8597</v>
+      </c>
+      <c r="R10" s="0" t="n">
+        <v>0.8581</v>
+      </c>
+      <c r="S10" s="0" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="T10" s="0" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="U10" s="0" t="n">
+        <v>0.8038</v>
+      </c>
+      <c r="V10" s="0" t="n">
+        <v>0.8689</v>
+      </c>
+      <c r="W10" s="0" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="X10" s="0" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="Y10" s="0" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="Z10" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="AA10" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AB10" s="0" t="n">
+        <v>0.8531</v>
+      </c>
+      <c r="AC10" s="0" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="AD10" s="0" t="n">
+        <v>0.8566</v>
+      </c>
+      <c r="AE10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="0" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="AG10" s="0" t="n">
+        <v>0.7981</v>
+      </c>
+      <c r="AH10" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AI10" s="0" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AJ10" s="0" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="AK10" s="0" t="n">
+        <v>0.693</v>
+      </c>
+      <c r="AL10" s="0" t="n">
+        <v>0.1809</v>
+      </c>
+      <c r="AM10" s="0" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="AN10" s="0" t="n">
+        <v>0.705</v>
+      </c>
+      <c r="AO10" s="0" t="n">
+        <v>0.5425</v>
+      </c>
+      <c r="AP10" s="0" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="AQ10" s="0" t="n">
+        <v>0.905</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <v>-0.0325</v>
+      </c>
+      <c r="J11" s="0" t="n">
+        <v>-0.0325</v>
+      </c>
+      <c r="K11" s="0" t="n">
+        <v>-0.2075</v>
+      </c>
+      <c r="L11" s="0" t="n">
+        <v>-0.4075</v>
+      </c>
+      <c r="M11" s="0" t="n">
+        <v>-0.2465</v>
+      </c>
+      <c r="N11" s="0" t="n">
+        <v>-0.6446</v>
+      </c>
+      <c r="O11" s="0" t="n">
+        <v>-0.1325</v>
+      </c>
+      <c r="P11" s="0" t="n">
+        <v>-0.6825</v>
+      </c>
+      <c r="Q11" s="0" t="n">
+        <v>-0.1403</v>
+      </c>
+      <c r="R11" s="0" t="n">
+        <v>-0.1419</v>
+      </c>
+      <c r="S11" s="0" t="n">
+        <v>-0.345</v>
+      </c>
+      <c r="T11" s="0" t="n">
+        <v>-0.395</v>
+      </c>
+      <c r="U11" s="0" t="n">
+        <v>-0.1962</v>
+      </c>
+      <c r="V11" s="0" t="n">
+        <v>-0.1311</v>
+      </c>
+      <c r="W11" s="0" t="n">
+        <v>-0.795</v>
+      </c>
+      <c r="X11" s="0" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="Y11" s="0" t="n">
+        <v>-0.445</v>
+      </c>
+      <c r="Z11" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="AA11" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AB11" s="0" t="n">
+        <v>-0.1469</v>
+      </c>
+      <c r="AC11" s="0" t="n">
+        <v>-0.208</v>
+      </c>
+      <c r="AD11" s="0" t="n">
+        <v>-0.1434</v>
+      </c>
+      <c r="AE11" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AF11" s="0" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="AG11" s="0" t="n">
+        <v>-0.2019</v>
+      </c>
+      <c r="AH11" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="AI11" s="0" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="AJ11" s="0" t="n">
+        <v>-0.031</v>
+      </c>
+      <c r="AK11" s="0" t="n">
+        <v>-0.307</v>
+      </c>
+      <c r="AL11" s="0" t="n">
+        <v>-0.8191</v>
+      </c>
+      <c r="AM11" s="0" t="n">
+        <v>-0.445</v>
+      </c>
+      <c r="AN11" s="0" t="n">
+        <v>-0.295</v>
+      </c>
+      <c r="AO11" s="0" t="n">
+        <v>-0.4575</v>
+      </c>
+      <c r="AP11" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="AQ11" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="I12" s="0" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="J12" s="0" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="K12" s="0" t="n">
+        <v>0.9738</v>
+      </c>
+      <c r="L12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="M12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="N12" s="0" t="n">
+        <v>0.9691</v>
+      </c>
+      <c r="O12" s="0" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="P12" s="0" t="n">
+        <v>0.9858</v>
+      </c>
+      <c r="Q12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="R12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="S12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="T12" s="0" t="n">
+        <v>0.9463</v>
+      </c>
+      <c r="U12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="V12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="W12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="X12" s="0" t="n">
+        <v>0.9871</v>
+      </c>
+      <c r="Y12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="Z12" s="0" t="n">
+        <v>0.9791</v>
+      </c>
+      <c r="AA12" s="0" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="AB12" s="0" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="AC12" s="0" t="n">
+        <v>0.9765</v>
+      </c>
+      <c r="AD12" s="0" t="n">
+        <v>0.9725</v>
+      </c>
+      <c r="AE12" s="0" t="n">
+        <v>0.8838</v>
+      </c>
+      <c r="AF12" s="0" t="n">
+        <v>0.9854</v>
+      </c>
+      <c r="AG12" s="0" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="AH12" s="0" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AI12" s="0" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="AJ12" s="0" t="n">
+        <v>0.9889</v>
+      </c>
+      <c r="AK12" s="0" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="AL12" s="0" t="n">
+        <v>0.9409</v>
+      </c>
+      <c r="AM12" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AN12" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="AO12" s="0" t="n">
+        <v>0.9637</v>
+      </c>
+      <c r="AP12" s="0" t="n">
+        <v>0.9894</v>
+      </c>
+      <c r="AQ12" s="0" t="n">
+        <v>0.9894</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="I13" s="0" t="n">
+        <v>-0.0102</v>
+      </c>
+      <c r="J13" s="0" t="n">
+        <v>-0.0102</v>
+      </c>
+      <c r="K13" s="0" t="n">
+        <v>-0.0262</v>
+      </c>
+      <c r="L13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="M13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="N13" s="0" t="n">
+        <v>-0.0309</v>
+      </c>
+      <c r="O13" s="0" t="n">
+        <v>-0.0102</v>
+      </c>
+      <c r="P13" s="0" t="n">
+        <v>-0.0143</v>
+      </c>
+      <c r="Q13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="R13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="S13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="T13" s="0" t="n">
+        <v>-0.0538</v>
+      </c>
+      <c r="U13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="V13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="W13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="X13" s="0" t="n">
+        <v>-0.0129</v>
+      </c>
+      <c r="Y13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="Z13" s="0" t="n">
+        <v>-0.0209</v>
+      </c>
+      <c r="AA13" s="0" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="AB13" s="0" t="n">
+        <v>-0.0164</v>
+      </c>
+      <c r="AC13" s="0" t="n">
+        <v>-0.0235</v>
+      </c>
+      <c r="AD13" s="0" t="n">
+        <v>-0.0275</v>
+      </c>
+      <c r="AE13" s="0" t="n">
+        <v>-0.1163</v>
+      </c>
+      <c r="AF13" s="0" t="n">
+        <v>-0.0146</v>
+      </c>
+      <c r="AG13" s="0" t="n">
+        <v>-0.083</v>
+      </c>
+      <c r="AH13" s="0" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AI13" s="0" t="n">
+        <v>-0.0102</v>
+      </c>
+      <c r="AJ13" s="0" t="n">
+        <v>-0.0111</v>
+      </c>
+      <c r="AK13" s="0" t="n">
+        <v>-0.0357</v>
+      </c>
+      <c r="AL13" s="0" t="n">
+        <v>-0.0591</v>
+      </c>
+      <c r="AM13" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="AN13" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="AO13" s="0" t="n">
+        <v>-0.0363</v>
+      </c>
+      <c r="AP13" s="0" t="n">
+        <v>-0.0106</v>
+      </c>
+      <c r="AQ13" s="0" t="n">
+        <v>-0.0106</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="I14" s="0" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="J14" s="0" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="K14" s="0" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="L14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="M14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="N14" s="0" t="n">
+        <v>0.6711</v>
+      </c>
+      <c r="O14" s="0" t="n">
+        <v>0.9765</v>
+      </c>
+      <c r="P14" s="0" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="Q14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="R14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="S14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="T14" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="U14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="V14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="W14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="X14" s="0" t="n">
+        <v>0.9675</v>
+      </c>
+      <c r="Y14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="Z14" s="0" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AA14" s="0" t="n">
+        <v>0.968</v>
+      </c>
+      <c r="AB14" s="0" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="AC14" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AD14" s="0" t="n">
+        <v>0.9593</v>
+      </c>
+      <c r="AE14" s="0" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AF14" s="0" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AG14" s="0" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="AH14" s="0" t="n">
+        <v>0.9741</v>
+      </c>
+      <c r="AI14" s="0" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="AJ14" s="0" t="n">
+        <v>0.9785</v>
+      </c>
+      <c r="AK14" s="0" t="n">
+        <v>0.9076</v>
+      </c>
+      <c r="AL14" s="0" t="n">
+        <v>0.6332</v>
+      </c>
+      <c r="AM14" s="0" t="n">
+        <v>0.7675</v>
+      </c>
+      <c r="AN14" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="AO14" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="AP14" s="0" t="n">
+        <v>0.9741</v>
+      </c>
+      <c r="AQ14" s="0" t="n">
+        <v>0.9741</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="I15" s="0" t="n">
+        <v>-0.0211</v>
+      </c>
+      <c r="J15" s="0" t="n">
+        <v>-0.0211</v>
+      </c>
+      <c r="K15" s="0" t="n">
+        <v>-0.0825</v>
+      </c>
+      <c r="L15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="M15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="N15" s="0" t="n">
+        <v>-0.3289</v>
+      </c>
+      <c r="O15" s="0" t="n">
+        <v>-0.0235</v>
+      </c>
+      <c r="P15" s="0" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="Q15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="R15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="S15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="T15" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="U15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="V15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="W15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="X15" s="0" t="n">
+        <v>-0.0325</v>
+      </c>
+      <c r="Y15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="Z15" s="0" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="AA15" s="0" t="n">
+        <v>-0.032</v>
+      </c>
+      <c r="AB15" s="0" t="n">
+        <v>-0.0825</v>
+      </c>
+      <c r="AC15" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AD15" s="0" t="n">
+        <v>-0.0407</v>
+      </c>
+      <c r="AE15" s="0" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="AF15" s="0" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="AG15" s="0" t="n">
+        <v>-0.0758</v>
+      </c>
+      <c r="AH15" s="0" t="n">
+        <v>-0.0259</v>
+      </c>
+      <c r="AI15" s="0" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="AJ15" s="0" t="n">
+        <v>-0.0215</v>
+      </c>
+      <c r="AK15" s="0" t="n">
+        <v>-0.0924</v>
+      </c>
+      <c r="AL15" s="0" t="n">
+        <v>-0.3668</v>
+      </c>
+      <c r="AM15" s="0" t="n">
+        <v>-0.2325</v>
+      </c>
+      <c r="AN15" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="AO15" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="AP15" s="0" t="n">
+        <v>-0.0259</v>
+      </c>
+      <c r="AQ15" s="0" t="n">
+        <v>-0.0259</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="I16" s="0" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J16" s="0" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K16" s="0" t="n">
+        <v>0.9637</v>
+      </c>
+      <c r="L16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="M16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="N16" s="0" t="n">
+        <v>0.5453</v>
+      </c>
+      <c r="O16" s="0" t="n">
+        <v>0.9779</v>
+      </c>
+      <c r="P16" s="0" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="Q16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="R16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="S16" s="0" t="n">
+        <v>0.9537</v>
+      </c>
+      <c r="T16" s="0" t="n">
+        <v>0.9138</v>
+      </c>
+      <c r="U16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="V16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="W16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="X16" s="0" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="Y16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="Z16" s="0" t="n">
+        <v>0.9513</v>
+      </c>
+      <c r="AA16" s="0" t="n">
+        <v>0.9637</v>
+      </c>
+      <c r="AB16" s="0" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="AC16" s="0" t="n">
+        <v>0.9791</v>
+      </c>
+      <c r="AD16" s="0" t="n">
+        <v>0.9792</v>
+      </c>
+      <c r="AE16" s="0" t="n">
+        <v>0.7275</v>
+      </c>
+      <c r="AF16" s="0" t="n">
+        <v>0.5025</v>
+      </c>
+      <c r="AG16" s="0" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="AH16" s="0" t="n">
+        <v>0.9712</v>
+      </c>
+      <c r="AI16" s="0" t="n">
+        <v>0.9872</v>
+      </c>
+      <c r="AJ16" s="0" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AK16" s="0" t="n">
+        <v>0.9594</v>
+      </c>
+      <c r="AL16" s="0" t="n">
+        <v>0.8839</v>
+      </c>
+      <c r="AM16" s="0" t="n">
+        <v>0.9487</v>
+      </c>
+      <c r="AN16" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="AO16" s="0" t="n">
+        <v>0.8525</v>
+      </c>
+      <c r="AP16" s="0" t="n">
+        <v>0.9851</v>
+      </c>
+      <c r="AQ16" s="0" t="n">
+        <v>0.9851</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="I17" s="0" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="J17" s="0" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="K17" s="0" t="n">
+        <v>-0.0362</v>
+      </c>
+      <c r="L17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="M17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="N17" s="0" t="n">
+        <v>-0.4547</v>
+      </c>
+      <c r="O17" s="0" t="n">
+        <v>-0.0221</v>
+      </c>
+      <c r="P17" s="0" t="n">
+        <v>-0.785</v>
+      </c>
+      <c r="Q17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="R17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="S17" s="0" t="n">
+        <v>-0.0462</v>
+      </c>
+      <c r="T17" s="0" t="n">
+        <v>-0.0862</v>
+      </c>
+      <c r="U17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="V17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="W17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="X17" s="0" t="n">
+        <v>-0.0825</v>
+      </c>
+      <c r="Y17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="Z17" s="0" t="n">
+        <v>-0.0488</v>
+      </c>
+      <c r="AA17" s="0" t="n">
+        <v>-0.0362</v>
+      </c>
+      <c r="AB17" s="0" t="n">
+        <v>-0.21</v>
+      </c>
+      <c r="AC17" s="0" t="n">
+        <v>-0.0209</v>
+      </c>
+      <c r="AD17" s="0" t="n">
+        <v>-0.0208</v>
+      </c>
+      <c r="AE17" s="0" t="n">
+        <v>-0.2725</v>
+      </c>
+      <c r="AF17" s="0" t="n">
+        <v>-0.4975</v>
+      </c>
+      <c r="AG17" s="0" t="n">
+        <v>-0.0308</v>
+      </c>
+      <c r="AH17" s="0" t="n">
+        <v>-0.0288</v>
+      </c>
+      <c r="AI17" s="0" t="n">
+        <v>-0.0127</v>
+      </c>
+      <c r="AJ17" s="0" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AK17" s="0" t="n">
+        <v>-0.0406</v>
+      </c>
+      <c r="AL17" s="0" t="n">
+        <v>-0.1161</v>
+      </c>
+      <c r="AM17" s="0" t="n">
+        <v>-0.0512</v>
+      </c>
+      <c r="AN17" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="AO17" s="0" t="n">
+        <v>-0.1475</v>
+      </c>
+      <c r="AP17" s="0" t="n">
+        <v>-0.0149</v>
+      </c>
+      <c r="AQ17" s="0" t="n">
+        <v>-0.0149</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="I18" s="0" t="n">
+        <v>0.9795</v>
+      </c>
+      <c r="J18" s="0" t="n">
+        <v>0.9795</v>
+      </c>
+      <c r="K18" s="0" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="M18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="N18" s="0" t="n">
+        <v>0.5153</v>
+      </c>
+      <c r="O18" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="P18" s="0" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="Q18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="R18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="S18" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="T18" s="0" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="U18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="V18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="W18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="X18" s="0" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="Y18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="Z18" s="0" t="n">
+        <v>0.6675</v>
+      </c>
+      <c r="AA18" s="0" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AB18" s="0" t="n">
+        <v>0.5175</v>
+      </c>
+      <c r="AC18" s="0" t="n">
+        <v>0.9775</v>
+      </c>
+      <c r="AD18" s="0" t="n">
+        <v>0.9496</v>
+      </c>
+      <c r="AE18" s="0" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="AF18" s="0" t="n">
+        <v>0.7925</v>
+      </c>
+      <c r="AG18" s="0" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="AH18" s="0" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="AI18" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AJ18" s="0" t="n">
+        <v>0.9741</v>
+      </c>
+      <c r="AK18" s="0" t="n">
+        <v>0.8273</v>
+      </c>
+      <c r="AL18" s="0" t="n">
+        <v>0.3911</v>
+      </c>
+      <c r="AM18" s="0" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="AN18" s="0" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="AO18" s="0" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="AP18" s="0" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="AQ18" s="0" t="n">
+        <v>0.9698</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="I19" s="0" t="n">
+        <v>-0.0205</v>
+      </c>
+      <c r="J19" s="0" t="n">
+        <v>-0.0205</v>
+      </c>
+      <c r="K19" s="0" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="L19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="M19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="N19" s="0" t="n">
+        <v>-0.4847</v>
+      </c>
+      <c r="O19" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="P19" s="0" t="n">
+        <v>-0.795</v>
+      </c>
+      <c r="Q19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="R19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="S19" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="T19" s="0" t="n">
+        <v>-0.345</v>
+      </c>
+      <c r="U19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="V19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="W19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="X19" s="0" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="Y19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="Z19" s="0" t="n">
+        <v>-0.3325</v>
+      </c>
+      <c r="AA19" s="0" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="AB19" s="0" t="n">
+        <v>-0.4825</v>
+      </c>
+      <c r="AC19" s="0" t="n">
+        <v>-0.0225</v>
+      </c>
+      <c r="AD19" s="0" t="n">
+        <v>-0.0504</v>
+      </c>
+      <c r="AE19" s="0" t="n">
+        <v>-0.795</v>
+      </c>
+      <c r="AF19" s="0" t="n">
+        <v>-0.2075</v>
+      </c>
+      <c r="AG19" s="0" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="AH19" s="0" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="AI19" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="AJ19" s="0" t="n">
+        <v>-0.0259</v>
+      </c>
+      <c r="AK19" s="0" t="n">
+        <v>-0.1727</v>
+      </c>
+      <c r="AL19" s="0" t="n">
+        <v>-0.6089</v>
+      </c>
+      <c r="AM19" s="0" t="n">
+        <v>-0.395</v>
+      </c>
+      <c r="AN19" s="0" t="n">
+        <v>-0.1825</v>
+      </c>
+      <c r="AO19" s="0" t="n">
+        <v>-0.395</v>
+      </c>
+      <c r="AP19" s="0" t="n">
+        <v>-0.0302</v>
+      </c>
+      <c r="AQ19" s="0" t="n">
+        <v>-0.0302</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="I20" s="0" t="n">
+        <v>0.9861</v>
+      </c>
+      <c r="J20" s="0" t="n">
+        <v>0.9861</v>
+      </c>
+      <c r="K20" s="0" t="n">
+        <v>0.9889</v>
+      </c>
+      <c r="L20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="M20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="N20" s="0" t="n">
+        <v>0.9839</v>
+      </c>
+      <c r="O20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="P20" s="0" t="n">
+        <v>0.9832</v>
+      </c>
+      <c r="Q20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="R20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="S20" s="0" t="n">
+        <v>0.9894</v>
+      </c>
+      <c r="T20" s="0" t="n">
+        <v>0.9762</v>
+      </c>
+      <c r="U20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="V20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="W20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="X20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="Y20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="Z20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="AA20" s="0" t="n">
+        <v>0.9897</v>
+      </c>
+      <c r="AB20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="AC20" s="0" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="AD20" s="0" t="n">
+        <v>0.9889</v>
+      </c>
+      <c r="AE20" s="0" t="n">
+        <v>0.9844</v>
+      </c>
+      <c r="AF20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="AG20" s="0" t="n">
+        <v>0.9845</v>
+      </c>
+      <c r="AH20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="AI20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="AJ20" s="0" t="n">
+        <v>0.9861</v>
+      </c>
+      <c r="AK20" s="0" t="n">
+        <v>0.9895</v>
+      </c>
+      <c r="AL20" s="0" t="n">
+        <v>0.9858</v>
+      </c>
+      <c r="AM20" s="0" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="AN20" s="0" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="AO20" s="0" t="n">
+        <v>0.9895</v>
+      </c>
+      <c r="AP20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="AQ20" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="I21" s="0" t="n">
+        <v>-0.0139</v>
+      </c>
+      <c r="J21" s="0" t="n">
+        <v>-0.0139</v>
+      </c>
+      <c r="K21" s="0" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="L21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="M21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="N21" s="0" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="O21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="P21" s="0" t="n">
+        <v>-0.0168</v>
+      </c>
+      <c r="Q21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="R21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="S21" s="0" t="n">
+        <v>-0.0106</v>
+      </c>
+      <c r="T21" s="0" t="n">
+        <v>-0.0238</v>
+      </c>
+      <c r="U21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="V21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="W21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="X21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="Y21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="Z21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="AA21" s="0" t="n">
+        <v>-0.0103</v>
+      </c>
+      <c r="AB21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="AC21" s="0" t="n">
+        <v>-0.1125</v>
+      </c>
+      <c r="AD21" s="0" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="AE21" s="0" t="n">
+        <v>-0.0156</v>
+      </c>
+      <c r="AF21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="AG21" s="0" t="n">
+        <v>-0.0155</v>
+      </c>
+      <c r="AH21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="AI21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="AJ21" s="0" t="n">
+        <v>-0.0139</v>
+      </c>
+      <c r="AK21" s="0" t="n">
+        <v>-0.0105</v>
+      </c>
+      <c r="AL21" s="0" t="n">
+        <v>-0.0142</v>
+      </c>
+      <c r="AM21" s="0" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="AN21" s="0" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="AO21" s="0" t="n">
+        <v>-0.0105</v>
+      </c>
+      <c r="AP21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="AQ21" s="0" t="n">
+        <v>-0.0101</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="I22" s="0" t="n">
+        <v>0.9795</v>
+      </c>
+      <c r="J22" s="0" t="n">
+        <v>0.9795</v>
+      </c>
+      <c r="K22" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="L22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="M22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="N22" s="0" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="O22" s="0" t="n">
+        <v>0.9772</v>
+      </c>
+      <c r="P22" s="0" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="Q22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="R22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="S22" s="0" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="T22" s="0" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="U22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="V22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="W22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="X22" s="0" t="n">
+        <v>0.9793</v>
+      </c>
+      <c r="Y22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="Z22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AA22" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AB22" s="0" t="n">
+        <v>0.9772</v>
+      </c>
+      <c r="AC22" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="AD22" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AE22" s="0" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="AF22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AG22" s="0" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="AH22" s="0" t="n">
+        <v>0.9793</v>
+      </c>
+      <c r="AI22" s="0" t="n">
+        <v>0.9798</v>
+      </c>
+      <c r="AJ22" s="0" t="n">
+        <v>0.9769</v>
+      </c>
+      <c r="AK22" s="0" t="n">
+        <v>0.9685</v>
+      </c>
+      <c r="AL22" s="0" t="n">
+        <v>0.8186</v>
+      </c>
+      <c r="AM22" s="0" t="n">
+        <v>0.7175</v>
+      </c>
+      <c r="AN22" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AO22" s="0" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="AP22" s="0" t="n">
+        <v>0.9793</v>
+      </c>
+      <c r="AQ22" s="0" t="n">
+        <v>0.9793</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E23" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="I23" s="0" t="n">
+        <v>-0.0205</v>
+      </c>
+      <c r="J23" s="0" t="n">
+        <v>-0.0205</v>
+      </c>
+      <c r="K23" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="L23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="M23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="N23" s="0" t="n">
+        <v>-0.1325</v>
+      </c>
+      <c r="O23" s="0" t="n">
+        <v>-0.0227</v>
+      </c>
+      <c r="P23" s="0" t="n">
+        <v>-0.345</v>
+      </c>
+      <c r="Q23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="R23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="S23" s="0" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="T23" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="U23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="V23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="W23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="X23" s="0" t="n">
+        <v>-0.0207</v>
+      </c>
+      <c r="Y23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="Z23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AA23" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="AB23" s="0" t="n">
+        <v>-0.0227</v>
+      </c>
+      <c r="AC23" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="AD23" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="AE23" s="0" t="n">
+        <v>-0.245</v>
+      </c>
+      <c r="AF23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AG23" s="0" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="AH23" s="0" t="n">
+        <v>-0.0207</v>
+      </c>
+      <c r="AI23" s="0" t="n">
+        <v>-0.0202</v>
+      </c>
+      <c r="AJ23" s="0" t="n">
+        <v>-0.0231</v>
+      </c>
+      <c r="AK23" s="0" t="n">
+        <v>-0.0315</v>
+      </c>
+      <c r="AL23" s="0" t="n">
+        <v>-0.1814</v>
+      </c>
+      <c r="AM23" s="0" t="n">
+        <v>-0.2825</v>
+      </c>
+      <c r="AN23" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AO23" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="AP23" s="0" t="n">
+        <v>-0.0207</v>
+      </c>
+      <c r="AQ23" s="0" t="n">
+        <v>-0.0207</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="0" t="s">
+        <v>273</v>
+      </c>
+      <c r="I24" s="0" t="n">
+        <v>0.9894</v>
+      </c>
+      <c r="J24" s="0" t="n">
+        <v>0.9894</v>
+      </c>
+      <c r="K24" s="0" t="n">
+        <v>0.9637</v>
+      </c>
+      <c r="L24" s="0" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="M24" s="0" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="N24" s="0" t="n">
+        <v>0.7591</v>
+      </c>
+      <c r="O24" s="0" t="n">
+        <v>0.9884</v>
+      </c>
+      <c r="P24" s="0" t="n">
+        <v>0.4275</v>
+      </c>
+      <c r="Q24" s="0" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="R24" s="0" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="S24" s="0" t="n">
+        <v>0.9337</v>
+      </c>
+      <c r="T24" s="0" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="U24" s="0" t="n">
+        <v>0.9842</v>
+      </c>
+      <c r="V24" s="0" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="W24" s="0" t="n">
+        <v>0.3025</v>
+      </c>
+      <c r="X24" s="0" t="n">
+        <v>0.9798</v>
+      </c>
+      <c r="Y24" s="0" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="Z24" s="0" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AA24" s="0" t="n">
+        <v>0.9831</v>
+      </c>
+      <c r="AB24" s="0" t="n">
+        <v>0.9787</v>
+      </c>
+      <c r="AC24" s="0" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="AD24" s="0" t="n">
+        <v>0.9818</v>
+      </c>
+      <c r="AE24" s="0" t="n">
+        <v>0.8975</v>
+      </c>
+      <c r="AF24" s="0" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="AG24" s="0" t="n">
+        <v>0.9625</v>
+      </c>
+      <c r="AH24" s="0" t="n">
+        <v>0.9899</v>
+      </c>
+      <c r="AI24" s="0" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AJ24" s="0" t="n">
+        <v>0.9859</v>
+      </c>
+      <c r="AK24" s="0" t="n">
+        <v>0.9087</v>
+      </c>
+      <c r="AL24" s="0" t="n">
+        <v>0.8075</v>
+      </c>
+      <c r="AM24" s="0" t="n">
+        <v>0.9587</v>
+      </c>
+      <c r="AN24" s="0" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AO24" s="0" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="AP24" s="0" t="n">
+        <v>0.9725</v>
+      </c>
+      <c r="AQ24" s="0" t="n">
+        <v>0.9725</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="I25" s="0" t="n">
+        <v>-0.0106</v>
+      </c>
+      <c r="J25" s="0" t="n">
+        <v>-0.0106</v>
+      </c>
+      <c r="K25" s="0" t="n">
+        <v>-0.0362</v>
+      </c>
+      <c r="L25" s="0" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="M25" s="0" t="n">
+        <v>-0.0775</v>
+      </c>
+      <c r="N25" s="0" t="n">
+        <v>-0.2409</v>
+      </c>
+      <c r="O25" s="0" t="n">
+        <v>-0.0116</v>
+      </c>
+      <c r="P25" s="0" t="n">
+        <v>-0.5725</v>
+      </c>
+      <c r="Q25" s="0" t="n">
+        <v>-0.0775</v>
+      </c>
+      <c r="R25" s="0" t="n">
+        <v>-0.0775</v>
+      </c>
+      <c r="S25" s="0" t="n">
+        <v>-0.0663</v>
+      </c>
+      <c r="T25" s="0" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="U25" s="0" t="n">
+        <v>-0.0157</v>
+      </c>
+      <c r="V25" s="0" t="n">
+        <v>-0.0775</v>
+      </c>
+      <c r="W25" s="0" t="n">
+        <v>-0.6975</v>
+      </c>
+      <c r="X25" s="0" t="n">
+        <v>-0.0203</v>
+      </c>
+      <c r="Y25" s="0" t="n">
+        <v>-0.0775</v>
+      </c>
+      <c r="Z25" s="0" t="n">
+        <v>-0.0625</v>
+      </c>
+      <c r="AA25" s="0" t="n">
+        <v>-0.0169</v>
+      </c>
+      <c r="AB25" s="0" t="n">
+        <v>-0.0213</v>
+      </c>
+      <c r="AC25" s="0" t="n">
+        <v>-0.0226</v>
+      </c>
+      <c r="AD25" s="0" t="n">
+        <v>-0.0182</v>
+      </c>
+      <c r="AE25" s="0" t="n">
+        <v>-0.1025</v>
+      </c>
+      <c r="AF25" s="0" t="n">
+        <v>-0.0688</v>
+      </c>
+      <c r="AG25" s="0" t="n">
+        <v>-0.0375</v>
+      </c>
+      <c r="AH25" s="0" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AI25" s="0" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AJ25" s="0" t="n">
+        <v>-0.0141</v>
+      </c>
+      <c r="AK25" s="0" t="n">
+        <v>-0.0913</v>
+      </c>
+      <c r="AL25" s="0" t="n">
+        <v>-0.1925</v>
+      </c>
+      <c r="AM25" s="0" t="n">
+        <v>-0.0413</v>
+      </c>
+      <c r="AN25" s="0" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AO25" s="0" t="n">
+        <v>-0.0312</v>
+      </c>
+      <c r="AP25" s="0" t="n">
+        <v>-0.0275</v>
+      </c>
+      <c r="AQ25" s="0" t="n">
+        <v>-0.0275</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="D26" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="0" t="s">
+        <v>273</v>
+      </c>
+      <c r="I26" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="J26" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="K26" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="L26" s="0" t="n">
+        <v>0.8925</v>
+      </c>
+      <c r="M26" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="N26" s="0" t="n">
+        <v>0.8043</v>
+      </c>
+      <c r="O26" s="0" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="P26" s="0" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="Q26" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="R26" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="S26" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="T26" s="0" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="U26" s="0" t="n">
+        <v>0.9675</v>
+      </c>
+      <c r="V26" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="W26" s="0" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="X26" s="0" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="Y26" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="Z26" s="0" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AA26" s="0" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AB26" s="0" t="n">
+        <v>0.9753</v>
+      </c>
+      <c r="AC26" s="0" t="n">
+        <v>0.8925</v>
+      </c>
+      <c r="AD26" s="0" t="n">
+        <v>0.9707</v>
+      </c>
+      <c r="AE26" s="0" t="n">
+        <v>0.8425</v>
+      </c>
+      <c r="AF26" s="0" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="AG26" s="0" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="AH26" s="0" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="AI26" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AJ26" s="0" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="AK26" s="0" t="n">
+        <v>0.9226</v>
+      </c>
+      <c r="AL26" s="0" t="n">
+        <v>0.6681</v>
+      </c>
+      <c r="AM26" s="0" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="AN26" s="0" t="n">
+        <v>0.7425</v>
+      </c>
+      <c r="AO26" s="0" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="AP26" s="0" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="AQ26" s="0" t="n">
+        <v>0.905</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="I27" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="J27" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="K27" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="L27" s="0" t="n">
+        <v>-0.1075</v>
+      </c>
+      <c r="M27" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="N27" s="0" t="n">
+        <v>-0.1957</v>
+      </c>
+      <c r="O27" s="0" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="P27" s="0" t="n">
+        <v>-0.645</v>
+      </c>
+      <c r="Q27" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="R27" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="S27" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="T27" s="0" t="n">
+        <v>-0.0825</v>
+      </c>
+      <c r="U27" s="0" t="n">
+        <v>-0.0325</v>
+      </c>
+      <c r="V27" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="W27" s="0" t="n">
+        <v>-0.1325</v>
+      </c>
+      <c r="X27" s="0" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="Y27" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="Z27" s="0" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="AA27" s="0" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="AB27" s="0" t="n">
+        <v>-0.0247</v>
+      </c>
+      <c r="AC27" s="0" t="n">
+        <v>-0.1075</v>
+      </c>
+      <c r="AD27" s="0" t="n">
+        <v>-0.0293</v>
+      </c>
+      <c r="AE27" s="0" t="n">
+        <v>-0.1575</v>
+      </c>
+      <c r="AF27" s="0" t="n">
+        <v>-0.0825</v>
+      </c>
+      <c r="AG27" s="0" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="AH27" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="AI27" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AJ27" s="0" t="n">
+        <v>-0.0575</v>
+      </c>
+      <c r="AK27" s="0" t="n">
+        <v>-0.0774</v>
+      </c>
+      <c r="AL27" s="0" t="n">
+        <v>-0.3319</v>
+      </c>
+      <c r="AM27" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="AN27" s="0" t="n">
+        <v>-0.2575</v>
+      </c>
+      <c r="AO27" s="0" t="n">
+        <v>-0.0825</v>
+      </c>
+      <c r="AP27" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+      <c r="AQ27" s="0" t="n">
+        <v>-0.095</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="42" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="0" t="s">
+        <v>277</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="I32" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="J32" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="K32" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="L32" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="M32" s="0" t="s">
+        <v>210</v>
+      </c>
+      <c r="N32" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="O32" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="P32" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q32" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="R32" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="S32" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="T32" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="U32" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="V32" s="0" t="s">
+        <v>219</v>
+      </c>
+      <c r="W32" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="X32" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="Y32" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="Z32" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA32" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="AB32" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="AC32" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="AD32" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="AE32" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF32" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="AG32" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="AH32" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="AI32" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="AJ32" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="AK32" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="AL32" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="AM32" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="AN32" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="AO32" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="AP32" s="0" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="H33" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="0" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K33" s="0" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="L33" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="M33" s="0" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="N33" s="0" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O33" s="0" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="P33" s="0" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="Q33" s="0" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="R33" s="0" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="S33" s="0" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="T33" s="0" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="U33" s="0" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="V33" s="0" t="n">
+        <v>66</v>
+      </c>
+      <c r="W33" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="X33" s="0" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="Y33" s="0" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="Z33" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA33" s="0" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AB33" s="0" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="AC33" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD33" s="0" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="AE33" s="0" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="AF33" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG33" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AH33" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AI33" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AJ33" s="0" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="AK33" s="0" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="AL33" s="0" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="AM33" s="0" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AN33" s="0" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="AO33" s="0" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AP33" s="0" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="H34" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="I34" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J34" s="0" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="K34" s="0" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="L34" s="0" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="M34" s="0" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="N34" s="0" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="O34" s="0" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="P34" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q34" s="0" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="R34" s="0" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="S34" s="0" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="T34" s="0" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="U34" s="0" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="V34" s="0" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="W34" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="X34" s="0" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="Y34" s="0" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="Z34" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AA34" s="0" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="AB34" s="0" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="AC34" s="0" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="AD34" s="0" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE34" s="0" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="AF34" s="0" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="AG34" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AH34" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AI34" s="0" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AJ34" s="0" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="AK34" s="0" t="n">
+        <v>81.9</v>
+      </c>
+      <c r="AL34" s="0" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="AM34" s="0" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="AN34" s="0" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="AO34" s="0" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AP34" s="0" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="0" t="s">
+        <v>281</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="H35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="0" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M35" s="0" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="N35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="P35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S35" s="0" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="T35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="U35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="V35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="W35" s="0" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="X35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Y35" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="Z35" s="0" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AA35" s="0" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AB35" s="0" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AC35" s="0" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AD35" s="0" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="AE35" s="0" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AF35" s="0" t="n">
+        <v>8.3</v>
+      </c>
+      <c r="AG35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI35" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AJ35" s="0" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AK35" s="0" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AL35" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AM35" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AN35" s="0" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AO35" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AP35" s="0" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="0" t="s">
+        <v>281</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="H36" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I36" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J36" s="0" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="K36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="L36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="M36" s="0" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="N36" s="0" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O36" s="0" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="P36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Q36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="R36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="S36" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="T36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="U36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="V36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="W36" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="X36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Y36" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z36" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="AA36" s="0" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="AB36" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AC36" s="0" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AD36" s="0" t="n">
+        <v>62</v>
+      </c>
+      <c r="AE36" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AF36" s="0" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="AG36" s="0" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AH36" s="0" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="AI36" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AJ36" s="0" t="n">
+        <v>9.2</v>
+      </c>
+      <c r="AK36" s="0" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="AL36" s="0" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="AM36" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="AN36" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="AO36" s="0" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AP36" s="0" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="0" t="s">
+        <v>282</v>
+      </c>
+      <c r="C37" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="H37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="0" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="K37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="L37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="M37" s="0" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="N37" s="0" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O37" s="0" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="P37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="R37" s="0" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="S37" s="0" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="T37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="U37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="V37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="W37" s="0" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="X37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Y37" s="0" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="Z37" s="0" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AA37" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="AB37" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AC37" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AD37" s="0" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="AE37" s="0" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="AF37" s="0" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AG37" s="0" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AH37" s="0" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AI37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ37" s="0" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AK37" s="0" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="AL37" s="0" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="AM37" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="AN37" s="0" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="AO37" s="0" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP37" s="0" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="0" t="s">
+        <v>282</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="H38" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I38" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J38" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="K38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="L38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="M38" s="0" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="N38" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="O38" s="0" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="P38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="Q38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="R38" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="S38" s="0" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="T38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="U38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="V38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="W38" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="X38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="Y38" s="0" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="Z38" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA38" s="0" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="AB38" s="0" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AC38" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD38" s="0" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="AE38" s="0" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="AF38" s="0" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="AG38" s="0" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AH38" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AI38" s="0" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AJ38" s="0" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="AK38" s="0" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="AL38" s="0" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="AM38" s="0" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="AN38" s="0" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="AO38" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP38" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="0" t="s">
+        <v>283</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="H39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J39" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="K39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M39" s="0" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" s="0" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="P39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Q39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="R39" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="S39" s="0" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="T39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="U39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="V39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="W39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="X39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Y39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Z39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB39" s="0" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="AC39" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AD39" s="0" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AE39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AF39" s="0" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AJ39" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AK39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AL39" s="0" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AM39" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AN39" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AO39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP39" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="0" t="s">
+        <v>283</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="H40" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="L40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="M40" s="0" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="N40" s="0" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O40" s="0" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="P40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="Q40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="R40" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="S40" s="0" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="T40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="U40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="V40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="W40" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="X40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="Y40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="Z40" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AA40" s="0" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AB40" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="AC40" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AD40" s="0" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="AE40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AF40" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AG40" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AH40" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI40" s="0" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AJ40" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="AK40" s="0" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="AL40" s="0" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="AM40" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AN40" s="0" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AO40" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AP40" s="0" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="0" t="s">
+        <v>284</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="H41" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I41" s="0" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J41" s="0" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="K41" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="L41" s="0" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="M41" s="0" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="N41" s="0" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O41" s="0" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="P41" s="0" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q41" s="0" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="R41" s="0" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="S41" s="0" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="T41" s="0" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="U41" s="0" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="V41" s="0" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="W41" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="X41" s="0" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Y41" s="0" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="Z41" s="0" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AA41" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AB41" s="0" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AC41" s="0" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD41" s="0" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="AE41" s="0" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="AF41" s="0" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="AG41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI41" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AJ41" s="0" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="AK41" s="0" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="AL41" s="0" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AM41" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN41" s="0" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AO41" s="0" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="AP41" s="0" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="0" t="s">
+        <v>284</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="H42" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I42" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J42" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K42" s="0" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="L42" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="M42" s="0" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="N42" s="0" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O42" s="0" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="P42" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="Q42" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="R42" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="S42" s="0" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="T42" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="U42" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="V42" s="0" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="W42" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="X42" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="Y42" s="0" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="Z42" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA42" s="0" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AB42" s="0" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="AC42" s="0" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AD42" s="0" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="AE42" s="0" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="AF42" s="0" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="AG42" s="0" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AH42" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AI42" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AJ42" s="0" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="AK42" s="0" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="AL42" s="0" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AM42" s="0" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="AN42" s="0" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="AO42" s="0" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AP42" s="0" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>